<commit_message>
fix(io): harden xlsx reader fidelity and limits
</commit_message>
<xml_diff>
--- a/tests/corpus/xlsx/l2_hidden_sheet.xlsx
+++ b/tests/corpus/xlsx/l2_hidden_sheet.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <bookViews>
+    <workbookView activeTab="1"/>
+  </bookViews>
   <sheets>
-    <sheet name="Visible" sheetId="1" r:id="rId1"/>
-    <sheet name="Hidden" sheetId="2" r:id="rId4" state="hidden"/>
+    <sheet name="Hidden" sheetId="1" r:id="rId1" state="hidden"/>
+    <sheet name="Visible" sheetId="2" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="LocalRate" localSheetId="1">Visible!$A$1</definedName>
+  </definedNames>
 </workbook>
 </file>
 

</xml_diff>